<commit_message>
run for 2024 pep vintage, update for insights 2025
</commit_message>
<xml_diff>
--- a/output_data/charts/0500000US39041.xlsx
+++ b/output_data/charts/0500000US39041.xlsx
@@ -167,10 +167,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$15</c:f>
+              <c:f>Sheet1!$A$2:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>2010</c:v>
                 </c:pt>
@@ -212,16 +212,19 @@
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$15</c:f>
+              <c:f>Sheet1!$B$2:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>4.386856562011033</c:v>
                 </c:pt>
@@ -253,16 +256,19 @@
                   <c:v>7.789081270737196</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8.16021118578214</c:v>
+                  <c:v>8.160362889357787</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>8.429967191185908</c:v>
+                  <c:v>8.430484763040885</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>8.934956693712863</c:v>
+                  <c:v>9.058711587256838</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>9.498955257386589</c:v>
+                  <c:v>9.751559733942903</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>10.42165687535194</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -292,10 +298,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$15</c:f>
+              <c:f>Sheet1!$A$2:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>2010</c:v>
                 </c:pt>
@@ -337,16 +343,19 @@
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$15</c:f>
+              <c:f>Sheet1!$C$2:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>3.348104663247942</c:v>
                 </c:pt>
@@ -378,16 +387,19 @@
                   <c:v>3.805632889668586</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.94532593439484</c:v>
+                  <c:v>3.946793578791794</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.173407687927622</c:v>
+                  <c:v>4.175704008965043</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4.472775752010807</c:v>
+                  <c:v>4.474732168029321</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4.67069022086377</c:v>
+                  <c:v>4.672756647130606</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.925913786003043</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -417,10 +429,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$15</c:f>
+              <c:f>Sheet1!$A$2:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>2010</c:v>
                 </c:pt>
@@ -462,16 +474,19 @@
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$15</c:f>
+              <c:f>Sheet1!$D$2:$D$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>2.115764587640052</c:v>
                 </c:pt>
@@ -503,16 +518,19 @@
                   <c:v>2.787365089050761</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.257484918620972</c:v>
+                  <c:v>3.258939775610935</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.311159515911823</c:v>
+                  <c:v>3.313993420814807</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.453466710223109</c:v>
+                  <c:v>3.472564843529744</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.502478025868173</c:v>
+                  <c:v>3.580083529553306</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.754317843725574</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -542,10 +560,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$15</c:f>
+              <c:f>Sheet1!$A$2:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>2010</c:v>
                 </c:pt>
@@ -587,16 +605,19 @@
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$15</c:f>
+              <c:f>Sheet1!$E$2:$E$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0.1541852735932021</c:v>
                 </c:pt>
@@ -628,16 +649,19 @@
                   <c:v>0.1849662484268335</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.1877620070085423</c:v>
+                  <c:v>0.1886950297915059</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.1898030567330375</c:v>
+                  <c:v>0.1902360553808336</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1968868915709455</c:v>
+                  <c:v>0.1955878206935438</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.1934068970280958</c:v>
+                  <c:v>0.1907773748345737</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.1891026449156602</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -667,10 +691,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$15</c:f>
+              <c:f>Sheet1!$A$2:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>2010</c:v>
                 </c:pt>
@@ -712,16 +736,19 @@
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$2:$F$15</c:f>
+              <c:f>Sheet1!$F$2:$F$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>1.576116130063844</c:v>
                 </c:pt>
@@ -753,16 +780,19 @@
                   <c:v>1.91401929750963</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.972430588475874</c:v>
+                  <c:v>1.971072958979745</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.051228748836326</c:v>
+                  <c:v>2.049669233271879</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.111015954018523</c:v>
+                  <c:v>2.104331124894277</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.189210658101504</c:v>
+                  <c:v>2.1767526597116</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.181404066127094</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -792,10 +822,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$15</c:f>
+              <c:f>Sheet1!$A$2:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>2010</c:v>
                 </c:pt>
@@ -837,16 +867,19 @@
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$2:$G$15</c:f>
+              <c:f>Sheet1!$G$2:$G$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>88.41897278344393</c:v>
                 </c:pt>
@@ -878,16 +911,19 @@
                   <c:v>83.51893520460699</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>82.47678536571763</c:v>
+                  <c:v>82.47413576746824</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>81.84443379940528</c:v>
+                  <c:v>81.83991251852655</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>80.83089799846375</c:v>
+                  <c:v>80.69407245559628</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>79.94525894075187</c:v>
+                  <c:v>79.62807005482702</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>78.5276047838767</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1006,13 +1042,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1428750</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1320,7 +1356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" style="1" customWidth="1"/>
@@ -1590,22 +1626,22 @@
         <v>2020</v>
       </c>
       <c r="B12" s="2">
-        <v>8.16021118578214</v>
+        <v>8.160362889357787</v>
       </c>
       <c r="C12" s="2">
-        <v>3.94532593439484</v>
+        <v>3.946793578791794</v>
       </c>
       <c r="D12" s="2">
-        <v>3.257484918620972</v>
+        <v>3.258939775610935</v>
       </c>
       <c r="E12" s="2">
-        <v>0.1877620070085423</v>
+        <v>0.1886950297915059</v>
       </c>
       <c r="F12" s="2">
-        <v>1.972430588475874</v>
+        <v>1.971072958979745</v>
       </c>
       <c r="G12" s="2">
-        <v>82.47678536571763</v>
+        <v>82.47413576746824</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1613,22 +1649,22 @@
         <v>2021</v>
       </c>
       <c r="B13" s="2">
-        <v>8.429967191185908</v>
+        <v>8.430484763040885</v>
       </c>
       <c r="C13" s="2">
-        <v>4.173407687927622</v>
+        <v>4.175704008965043</v>
       </c>
       <c r="D13" s="2">
-        <v>3.311159515911823</v>
+        <v>3.313993420814807</v>
       </c>
       <c r="E13" s="2">
-        <v>0.1898030567330375</v>
+        <v>0.1902360553808336</v>
       </c>
       <c r="F13" s="2">
-        <v>2.051228748836326</v>
+        <v>2.049669233271879</v>
       </c>
       <c r="G13" s="2">
-        <v>81.84443379940528</v>
+        <v>81.83991251852655</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1636,22 +1672,22 @@
         <v>2022</v>
       </c>
       <c r="B14" s="2">
-        <v>8.934956693712863</v>
+        <v>9.058711587256838</v>
       </c>
       <c r="C14" s="2">
-        <v>4.472775752010807</v>
+        <v>4.474732168029321</v>
       </c>
       <c r="D14" s="2">
-        <v>3.453466710223109</v>
+        <v>3.472564843529744</v>
       </c>
       <c r="E14" s="2">
-        <v>0.1968868915709455</v>
+        <v>0.1955878206935438</v>
       </c>
       <c r="F14" s="2">
-        <v>2.111015954018523</v>
+        <v>2.104331124894277</v>
       </c>
       <c r="G14" s="2">
-        <v>80.83089799846375</v>
+        <v>80.69407245559628</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1659,22 +1695,45 @@
         <v>2023</v>
       </c>
       <c r="B15" s="2">
-        <v>9.498955257386589</v>
+        <v>9.751559733942903</v>
       </c>
       <c r="C15" s="2">
-        <v>4.67069022086377</v>
+        <v>4.672756647130606</v>
       </c>
       <c r="D15" s="2">
-        <v>3.502478025868173</v>
+        <v>3.580083529553306</v>
       </c>
       <c r="E15" s="2">
-        <v>0.1934068970280958</v>
+        <v>0.1907773748345737</v>
       </c>
       <c r="F15" s="2">
-        <v>2.189210658101504</v>
+        <v>2.1767526597116</v>
       </c>
       <c r="G15" s="2">
-        <v>79.94525894075187</v>
+        <v>79.62807005482702</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="3">
+        <v>2024</v>
+      </c>
+      <c r="B16" s="2">
+        <v>10.42165687535194</v>
+      </c>
+      <c r="C16" s="2">
+        <v>4.925913786003043</v>
+      </c>
+      <c r="D16" s="2">
+        <v>3.754317843725574</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.1891026449156602</v>
+      </c>
+      <c r="F16" s="2">
+        <v>2.181404066127094</v>
+      </c>
+      <c r="G16" s="2">
+        <v>78.5276047838767</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update script to account for schema change in input data. Changes to outputs are incidental.
</commit_message>
<xml_diff>
--- a/output_data/charts/0500000US39041.xlsx
+++ b/output_data/charts/0500000US39041.xlsx
@@ -226,34 +226,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>4.386856562011033</c:v>
+                  <c:v>4.386090154712477</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.610155445056668</c:v>
+                  <c:v>4.602458901615929</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.756833706699625</c:v>
+                  <c:v>4.744737118154664</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.059150071411248</c:v>
+                  <c:v>5.042615168842378</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.414212571645514</c:v>
+                  <c:v>5.389041385135135</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.83192166260381</c:v>
+                  <c:v>5.794995630613627</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.297545608330547</c:v>
+                  <c:v>6.218297285233129</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6.767847999323911</c:v>
+                  <c:v>6.639119828744959</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7.230687567872918</c:v>
+                  <c:v>7.070519915549683</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>7.789081270737196</c:v>
+                  <c:v>7.571100073143796</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>8.160362889357787</c:v>
@@ -357,34 +357,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>3.348104663247942</c:v>
+                  <c:v>3.341538215523789</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.360323433230301</c:v>
+                  <c:v>3.351163637382025</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.337122173543595</c:v>
+                  <c:v>3.31977010605818</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.333962111617128</c:v>
+                  <c:v>3.302945301542777</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.320344425754947</c:v>
+                  <c:v>3.281777871621622</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.342560839565343</c:v>
+                  <c:v>3.302635593176518</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.439491091054588</c:v>
+                  <c:v>3.397009292699753</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.578796661314297</c:v>
+                  <c:v>3.53064170856773</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.682060122621709</c:v>
+                  <c:v>3.640822854245189</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.805632889668586</c:v>
+                  <c:v>3.755671034578371</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>3.946793578791794</c:v>
@@ -488,34 +488,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>2.115764587640052</c:v>
+                  <c:v>2.115374730866538</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.17936657259329</c:v>
+                  <c:v>2.173803455905005</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.279373627465045</c:v>
+                  <c:v>2.270782379214584</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.333665687569054</c:v>
+                  <c:v>2.324954148236056</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.389150483261183</c:v>
+                  <c:v>2.380701013513514</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.416539271991075</c:v>
+                  <c:v>2.406006484272794</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.542012337800468</c:v>
+                  <c:v>2.536217181349674</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.575600153114234</c:v>
+                  <c:v>2.581271469109374</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.704690109911516</c:v>
+                  <c:v>2.712942059866108</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.787365089050761</c:v>
+                  <c:v>2.801455226913093</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>3.258939775610935</c:v>
@@ -619,34 +619,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.1541852735932021</c:v>
+                  <c:v>0.1541984820016105</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.162948528423599</c:v>
+                  <c:v>0.1624331363598174</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1677389452310273</c:v>
+                  <c:v>0.1667338386877716</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.18054919291816</c:v>
+                  <c:v>0.1796310281583774</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1824423013039879</c:v>
+                  <c:v>0.1805320945945946</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.1750816014543652</c:v>
+                  <c:v>0.1732241934733261</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.1757478145480698</c:v>
+                  <c:v>0.1739844986405876</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.1779704409988218</c:v>
+                  <c:v>0.1762333847762234</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1821307348049886</c:v>
+                  <c:v>0.1804077214504781</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.1849662484268335</c:v>
+                  <c:v>0.1830985242163335</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0.1886950297915059</c:v>
@@ -750,34 +750,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.576116130063844</c:v>
+                  <c:v>1.576251149349796</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.621645836133136</c:v>
+                  <c:v>1.620410563755006</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.670768178156417</c:v>
+                  <c:v>1.666786288074114</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.724110054164758</c:v>
+                  <c:v>1.717553134102924</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.768530284894727</c:v>
+                  <c:v>1.758340371621621</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.812275337768045</c:v>
+                  <c:v>1.799980350688501</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.839021079608189</c:v>
+                  <c:v>1.831148804934464</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.901499823520931</c:v>
+                  <c:v>1.891770797032907</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.938669666467005</c:v>
+                  <c:v>1.924023969847531</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.91401929750963</c:v>
+                  <c:v>1.893611630341768</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>1.971072958979745</c:v>
@@ -881,34 +881,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>88.41897278344393</c:v>
+                  <c:v>88.42654726754579</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>88.06556018456301</c:v>
+                  <c:v>88.08973030498221</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>87.78816336890429</c:v>
+                  <c:v>87.83119026981069</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>87.36856288231965</c:v>
+                  <c:v>87.43230121911749</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>86.92531993313965</c:v>
+                  <c:v>87.00960726351352</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>86.42162128661735</c:v>
+                  <c:v>86.52315774777523</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>85.70618206865814</c:v>
+                  <c:v>85.8433429371424</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>84.9982849217278</c:v>
+                  <c:v>85.18096281176881</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>84.26176179832187</c:v>
+                  <c:v>84.47128347904102</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>83.51893520460699</c:v>
+                  <c:v>83.79506351080663</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>82.47413576746824</c:v>
@@ -1396,22 +1396,22 @@
         <v>2010</v>
       </c>
       <c r="B2" s="2">
-        <v>4.386856562011033</v>
+        <v>4.386090154712477</v>
       </c>
       <c r="C2" s="2">
-        <v>3.348104663247942</v>
+        <v>3.341538215523789</v>
       </c>
       <c r="D2" s="2">
-        <v>2.115764587640052</v>
+        <v>2.115374730866538</v>
       </c>
       <c r="E2" s="2">
-        <v>0.1541852735932021</v>
+        <v>0.1541984820016105</v>
       </c>
       <c r="F2" s="2">
-        <v>1.576116130063844</v>
+        <v>1.576251149349796</v>
       </c>
       <c r="G2" s="2">
-        <v>88.41897278344393</v>
+        <v>88.42654726754579</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1419,22 +1419,22 @@
         <v>2011</v>
       </c>
       <c r="B3" s="2">
-        <v>4.610155445056668</v>
+        <v>4.602458901615929</v>
       </c>
       <c r="C3" s="2">
-        <v>3.360323433230301</v>
+        <v>3.351163637382025</v>
       </c>
       <c r="D3" s="2">
-        <v>2.17936657259329</v>
+        <v>2.173803455905005</v>
       </c>
       <c r="E3" s="2">
-        <v>0.162948528423599</v>
+        <v>0.1624331363598174</v>
       </c>
       <c r="F3" s="2">
-        <v>1.621645836133136</v>
+        <v>1.620410563755006</v>
       </c>
       <c r="G3" s="2">
-        <v>88.06556018456301</v>
+        <v>88.08973030498221</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1442,22 +1442,22 @@
         <v>2012</v>
       </c>
       <c r="B4" s="2">
-        <v>4.756833706699625</v>
+        <v>4.744737118154664</v>
       </c>
       <c r="C4" s="2">
-        <v>3.337122173543595</v>
+        <v>3.31977010605818</v>
       </c>
       <c r="D4" s="2">
-        <v>2.279373627465045</v>
+        <v>2.270782379214584</v>
       </c>
       <c r="E4" s="2">
-        <v>0.1677389452310273</v>
+        <v>0.1667338386877716</v>
       </c>
       <c r="F4" s="2">
-        <v>1.670768178156417</v>
+        <v>1.666786288074114</v>
       </c>
       <c r="G4" s="2">
-        <v>87.78816336890429</v>
+        <v>87.83119026981069</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1465,22 +1465,22 @@
         <v>2013</v>
       </c>
       <c r="B5" s="2">
-        <v>5.059150071411248</v>
+        <v>5.042615168842378</v>
       </c>
       <c r="C5" s="2">
-        <v>3.333962111617128</v>
+        <v>3.302945301542777</v>
       </c>
       <c r="D5" s="2">
-        <v>2.333665687569054</v>
+        <v>2.324954148236056</v>
       </c>
       <c r="E5" s="2">
-        <v>0.18054919291816</v>
+        <v>0.1796310281583774</v>
       </c>
       <c r="F5" s="2">
-        <v>1.724110054164758</v>
+        <v>1.717553134102924</v>
       </c>
       <c r="G5" s="2">
-        <v>87.36856288231965</v>
+        <v>87.43230121911749</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1488,22 +1488,22 @@
         <v>2014</v>
       </c>
       <c r="B6" s="2">
-        <v>5.414212571645514</v>
+        <v>5.389041385135135</v>
       </c>
       <c r="C6" s="2">
-        <v>3.320344425754947</v>
+        <v>3.281777871621622</v>
       </c>
       <c r="D6" s="2">
-        <v>2.389150483261183</v>
+        <v>2.380701013513514</v>
       </c>
       <c r="E6" s="2">
-        <v>0.1824423013039879</v>
+        <v>0.1805320945945946</v>
       </c>
       <c r="F6" s="2">
-        <v>1.768530284894727</v>
+        <v>1.758340371621621</v>
       </c>
       <c r="G6" s="2">
-        <v>86.92531993313965</v>
+        <v>87.00960726351352</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1511,22 +1511,22 @@
         <v>2015</v>
       </c>
       <c r="B7" s="2">
-        <v>5.83192166260381</v>
+        <v>5.794995630613627</v>
       </c>
       <c r="C7" s="2">
-        <v>3.342560839565343</v>
+        <v>3.302635593176518</v>
       </c>
       <c r="D7" s="2">
-        <v>2.416539271991075</v>
+        <v>2.406006484272794</v>
       </c>
       <c r="E7" s="2">
-        <v>0.1750816014543652</v>
+        <v>0.1732241934733261</v>
       </c>
       <c r="F7" s="2">
-        <v>1.812275337768045</v>
+        <v>1.799980350688501</v>
       </c>
       <c r="G7" s="2">
-        <v>86.42162128661735</v>
+        <v>86.52315774777523</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1534,22 +1534,22 @@
         <v>2016</v>
       </c>
       <c r="B8" s="2">
-        <v>6.297545608330547</v>
+        <v>6.218297285233129</v>
       </c>
       <c r="C8" s="2">
-        <v>3.439491091054588</v>
+        <v>3.397009292699753</v>
       </c>
       <c r="D8" s="2">
-        <v>2.542012337800468</v>
+        <v>2.536217181349674</v>
       </c>
       <c r="E8" s="2">
-        <v>0.1757478145480698</v>
+        <v>0.1739844986405876</v>
       </c>
       <c r="F8" s="2">
-        <v>1.839021079608189</v>
+        <v>1.831148804934464</v>
       </c>
       <c r="G8" s="2">
-        <v>85.70618206865814</v>
+        <v>85.8433429371424</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1557,22 +1557,22 @@
         <v>2017</v>
       </c>
       <c r="B9" s="2">
-        <v>6.767847999323911</v>
+        <v>6.639119828744959</v>
       </c>
       <c r="C9" s="2">
-        <v>3.578796661314297</v>
+        <v>3.53064170856773</v>
       </c>
       <c r="D9" s="2">
-        <v>2.575600153114234</v>
+        <v>2.581271469109374</v>
       </c>
       <c r="E9" s="2">
-        <v>0.1779704409988218</v>
+        <v>0.1762333847762234</v>
       </c>
       <c r="F9" s="2">
-        <v>1.901499823520931</v>
+        <v>1.891770797032907</v>
       </c>
       <c r="G9" s="2">
-        <v>84.9982849217278</v>
+        <v>85.18096281176881</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1580,22 +1580,22 @@
         <v>2018</v>
       </c>
       <c r="B10" s="2">
-        <v>7.230687567872918</v>
+        <v>7.070519915549683</v>
       </c>
       <c r="C10" s="2">
-        <v>3.682060122621709</v>
+        <v>3.640822854245189</v>
       </c>
       <c r="D10" s="2">
-        <v>2.704690109911516</v>
+        <v>2.712942059866108</v>
       </c>
       <c r="E10" s="2">
-        <v>0.1821307348049886</v>
+        <v>0.1804077214504781</v>
       </c>
       <c r="F10" s="2">
-        <v>1.938669666467005</v>
+        <v>1.924023969847531</v>
       </c>
       <c r="G10" s="2">
-        <v>84.26176179832187</v>
+        <v>84.47128347904102</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1603,22 +1603,22 @@
         <v>2019</v>
       </c>
       <c r="B11" s="2">
-        <v>7.789081270737196</v>
+        <v>7.571100073143796</v>
       </c>
       <c r="C11" s="2">
-        <v>3.805632889668586</v>
+        <v>3.755671034578371</v>
       </c>
       <c r="D11" s="2">
-        <v>2.787365089050761</v>
+        <v>2.801455226913093</v>
       </c>
       <c r="E11" s="2">
-        <v>0.1849662484268335</v>
+        <v>0.1830985242163335</v>
       </c>
       <c r="F11" s="2">
-        <v>1.91401929750963</v>
+        <v>1.893611630341768</v>
       </c>
       <c r="G11" s="2">
-        <v>83.51893520460699</v>
+        <v>83.79506351080663</v>
       </c>
     </row>
     <row r="12" spans="1:7">

</xml_diff>